<commit_message>
Whiteboard as at 21Sep
</commit_message>
<xml_diff>
--- a/whiteboard.xlsx
+++ b/whiteboard.xlsx
@@ -8,22 +8,28 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\BLaptop\Kvaluent\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C889C48A-40C8-4A5A-92CA-56342B71CAC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{130177F4-1B48-4EFD-854D-FC8CDA4FAA61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{00843BC8-B95A-4820-BE6A-899021419895}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="7" xr2:uid="{00843BC8-B95A-4820-BE6A-899021419895}"/>
   </bookViews>
   <sheets>
     <sheet name="Day9" sheetId="1" r:id="rId1"/>
     <sheet name="Day10" sheetId="10" r:id="rId2"/>
-    <sheet name="Day3" sheetId="2" r:id="rId3"/>
-    <sheet name="TOC" sheetId="3" r:id="rId4"/>
-    <sheet name="Day4" sheetId="4" r:id="rId5"/>
-    <sheet name="Sheet3" sheetId="9" r:id="rId6"/>
-    <sheet name="Day5" sheetId="5" r:id="rId7"/>
-    <sheet name="Day6" sheetId="6" r:id="rId8"/>
-    <sheet name="Day7" sheetId="7" r:id="rId9"/>
-    <sheet name="Day8" sheetId="8" r:id="rId10"/>
+    <sheet name="Day12-MidEval" sheetId="11" r:id="rId3"/>
+    <sheet name="Day13" sheetId="12" r:id="rId4"/>
+    <sheet name="Day3" sheetId="2" r:id="rId5"/>
+    <sheet name="TOC" sheetId="3" r:id="rId6"/>
+    <sheet name="Day4" sheetId="4" r:id="rId7"/>
+    <sheet name="Day19DB" sheetId="9" r:id="rId8"/>
+    <sheet name="Day5" sheetId="5" r:id="rId9"/>
+    <sheet name="Day6" sheetId="6" r:id="rId10"/>
+    <sheet name="Day7" sheetId="7" r:id="rId11"/>
+    <sheet name="Day8" sheetId="8" r:id="rId12"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Day10'!$A$30:$Q$92</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Day12-MidEval'!$A$24:$G$33</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -43,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="675" uniqueCount="593">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1067" uniqueCount="898">
   <si>
     <t>Login use case</t>
   </si>
@@ -5629,13 +5635,928 @@
   </si>
   <si>
     <t>Hands on day 9 - classes evaluation</t>
+  </si>
+  <si>
+    <t>REQUEST ERROR: https://example.com/broken-test-page-019 --&gt; Error: apiRequestContext.get: getaddrinfo ENOTFOUND example.com</t>
+  </si>
+  <si>
+    <t>Call log:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  - → GET https://example.com/broken-test-page-019</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    - user-agent: Mozilla/5.0 (Windows NT 10.0; Win64; x64) AppleWebKit/537.36 (KHTML, like Gecko) Chrome/151.0.7922.34 Safari/537.36</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    - accept: */*</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    - accept-encoding: gzip,deflate,br</t>
+  </si>
+  <si>
+    <t>REQUEST ERROR: https://example.com/broken-test-page-020 --&gt; Error: apiRequestContext.get: getaddrinfo ENOTFOUND example.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  - → GET https://example.com/broken-test-page-020</t>
+  </si>
+  <si>
+    <t>Sc1</t>
+  </si>
+  <si>
+    <t>un</t>
+  </si>
+  <si>
+    <t>pw</t>
+  </si>
+  <si>
+    <t>right</t>
+  </si>
+  <si>
+    <t>success</t>
+  </si>
+  <si>
+    <t>exp result</t>
+  </si>
+  <si>
+    <t>actual</t>
+  </si>
+  <si>
+    <t>sc2</t>
+  </si>
+  <si>
+    <t>wrong</t>
+  </si>
+  <si>
+    <t>sc3</t>
+  </si>
+  <si>
+    <t>login use case</t>
+  </si>
+  <si>
+    <t>db server down</t>
+  </si>
+  <si>
+    <t>security issue</t>
+  </si>
+  <si>
+    <t>session is getting carried over.</t>
+  </si>
+  <si>
+    <t>Most unlikely</t>
+  </si>
+  <si>
+    <t>notify db team to inform for retest</t>
+  </si>
+  <si>
+    <t>abcdefghijklmnop</t>
+  </si>
+  <si>
+    <t>somepassword</t>
+  </si>
+  <si>
+    <t>registration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">client end </t>
+  </si>
+  <si>
+    <t xml:space="preserve">long names cannot be entered in username box </t>
+  </si>
+  <si>
+    <t>sc4</t>
+  </si>
+  <si>
+    <t>right-with long names</t>
+  </si>
+  <si>
+    <t>type</t>
+  </si>
+  <si>
+    <t>2bhk</t>
+  </si>
+  <si>
+    <t>location</t>
+  </si>
+  <si>
+    <t>city</t>
+  </si>
+  <si>
+    <t>bangalore</t>
+  </si>
+  <si>
+    <t>banashankari</t>
+  </si>
+  <si>
+    <t>bhanashankari</t>
+  </si>
+  <si>
+    <t>exp</t>
+  </si>
+  <si>
+    <t>exp:120</t>
+  </si>
+  <si>
+    <t>no of houses: 120</t>
+  </si>
+  <si>
+    <t>Total links found: 50</t>
+  </si>
+  <si>
+    <t>VALID: https://www.google.com --&gt; 200 Ok for link text: Google</t>
+  </si>
+  <si>
+    <t>VALID: https://www.microsoft.com --&gt; 200 Ok for link text: Microsoft</t>
+  </si>
+  <si>
+    <t>VALID: https://www.apple.com --&gt; 200 Ok for link text: Apple</t>
+  </si>
+  <si>
+    <t>VALID: https://www.amazon.com --&gt; 202 Ok for link text: Amazon</t>
+  </si>
+  <si>
+    <t>VALID: https://www.wikipedia.org --&gt; 200 Ok for link text: Wikipedia</t>
+  </si>
+  <si>
+    <t>VALID: https://www.github.com --&gt; 200 Ok for link text: GitHub</t>
+  </si>
+  <si>
+    <t>VALID: https://www.linkedin.com --&gt; 200 Ok for link text: LinkedIn</t>
+  </si>
+  <si>
+    <t>VALID: https://www.youtube.com --&gt; 200 Ok for link text: YouTube</t>
+  </si>
+  <si>
+    <t>VALID: https://www.mozilla.org --&gt; 200 Ok for link text: Mozilla</t>
+  </si>
+  <si>
+    <t>VALID: https://www.python.org --&gt; 200 Ok for link text: Python</t>
+  </si>
+  <si>
+    <t>CLIENT ERROR: https://www.oracle.com --&gt; 403 for link text: Oracle</t>
+  </si>
+  <si>
+    <t>VALID: https://www.ibm.com --&gt; 200 Ok for link text: IBM</t>
+  </si>
+  <si>
+    <t>VALID: https://www.w3.org --&gt; 200 Ok for link text: W3C</t>
+  </si>
+  <si>
+    <t>VALID: https://playwright.dev --&gt; 200 Ok for link text: Playwright</t>
+  </si>
+  <si>
+    <t>VALID: https://www.typescriptlang.org --&gt; 200 Ok for link text: TypeScript</t>
+  </si>
+  <si>
+    <t>VALID: https://nodejs.org --&gt; 200 Ok for link text: Node.js</t>
+  </si>
+  <si>
+    <t>CLIENT ERROR: https://www.npmjs.com --&gt; 403 for link text: NPM</t>
+  </si>
+  <si>
+    <t>VALID: https://developer.mozilla.org --&gt; 200 Ok for link text: MDN Web Docs</t>
+  </si>
+  <si>
+    <t>CLIENT ERROR: https://stackoverflow.com --&gt; 403 for link text: Stack Overflow</t>
+  </si>
+  <si>
+    <t>VALID: https://www.selenium.dev --&gt; 200 Ok for link text: Selenium</t>
+  </si>
+  <si>
+    <t>result</t>
+  </si>
+  <si>
+    <t>BROKEN LINK: 404 for link text: Broken Google Link</t>
+  </si>
+  <si>
+    <t>BROKEN LINK: 404 for link text: Broken Microsoft Link</t>
+  </si>
+  <si>
+    <t>BROKEN LINK: 404 for link text: Broken Apple Link</t>
+  </si>
+  <si>
+    <t>BROKEN LINK: 404 for link text: Broken Amazon Link</t>
+  </si>
+  <si>
+    <t>CLIENT ERROR: https://www.wikipedia.org/non-existent-page-005 --&gt; 429 for link text: Broken Wikipedia Link</t>
+  </si>
+  <si>
+    <t>BROKEN LINK: 404 for link text: Broken GitHub Link</t>
+  </si>
+  <si>
+    <t>BROKEN LINK: 404 for link text: Broken YouTube Link</t>
+  </si>
+  <si>
+    <t>BROKEN LINK: 404 for link text: Broken Mozilla Link</t>
+  </si>
+  <si>
+    <t>BROKEN LINK: 404 for link text: Broken Python Link</t>
+  </si>
+  <si>
+    <t>BROKEN LINK: 404 for link text: Broken IBM Link</t>
+  </si>
+  <si>
+    <t>BROKEN LINK: 404 for link text: Broken W3C Link</t>
+  </si>
+  <si>
+    <t>BROKEN LINK: 404 for link text: Broken Playwright Link</t>
+  </si>
+  <si>
+    <t>BROKEN LINK: 404 for link text: Broken TypeScript Link</t>
+  </si>
+  <si>
+    <t>BROKEN LINK: 404 for link text: Broken Node.js Link</t>
+  </si>
+  <si>
+    <t>CLIENT ERROR: https://www.npmjs.com/non-existent-page-015 --&gt; 403 for link text: Broken NPM Link</t>
+  </si>
+  <si>
+    <t>BROKEN LINK: 404 for link text: Broken MDN Link</t>
+  </si>
+  <si>
+    <t>CLIENT ERROR: https://stackoverflow.com/non-existent-page-017 --&gt; 403 for link text: Broken Stack Overflow Link</t>
+  </si>
+  <si>
+    <t>BROKEN LINK: 404 for link text: Broken Selenium Link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> for link text: Broken Example Link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> for link text: Another Broken Example Link</t>
+  </si>
+  <si>
+    <t>VALID: https://httpbin.org/status/200 --&gt; 200 Ok for link text: HTTP 200 - Valid</t>
+  </si>
+  <si>
+    <t>VALID: https://httpbin.org/status/201 --&gt; 201 Ok for link text: HTTP 201 - Valid</t>
+  </si>
+  <si>
+    <t>VALID: https://httpbin.org/status/204 --&gt; 204 Ok for link text: HTTP 204 - Valid</t>
+  </si>
+  <si>
+    <t>VALID: https://httpbin.org/status/301 --&gt; 200 Ok for link text: HTTP 301 - Redirect</t>
+  </si>
+  <si>
+    <t>VALID: https://httpbin.org/status/302 --&gt; 200 Ok for link text: HTTP 302 - Redirect</t>
+  </si>
+  <si>
+    <t>CLIENT ERROR: https://httpbin.org/status/400 --&gt; 400 for link text: HTTP 400 - Bad Request</t>
+  </si>
+  <si>
+    <t>CLIENT ERROR: https://httpbin.org/status/401 --&gt; 401 for link text: HTTP 401 - Unauthorized</t>
+  </si>
+  <si>
+    <t>CLIENT ERROR: https://httpbin.org/status/403 --&gt; 403 for link text: HTTP 403 - Forbidden</t>
+  </si>
+  <si>
+    <t>BROKEN LINK: 404 for link text: HTTP 404 - Not Found</t>
+  </si>
+  <si>
+    <t>SERVER ERROR: https://httpbin.org/status/500 --&gt; 500 for link text: HTTP 500 - Server Error</t>
+  </si>
+  <si>
+    <t>KRISHNAN Arunima</t>
+  </si>
+  <si>
+    <t>Organiser</t>
+  </si>
+  <si>
+    <t>Asmita</t>
+  </si>
+  <si>
+    <t>absent</t>
+  </si>
+  <si>
+    <t>family grievance</t>
+  </si>
+  <si>
+    <t>Evaluation  - Playwright midway tasks</t>
+  </si>
+  <si>
+    <t>Requirement - As given on 4 Sep Friday</t>
+  </si>
+  <si>
+    <t>1. include a smoke test in the same orangehome.spec.ts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     Check if Login heading is present in the web page</t>
+  </si>
+  <si>
+    <t>2. Simulate a error condition in the script for trace viewer  - npx playwright test &lt;spec filename&gt; --trace on</t>
+  </si>
+  <si>
+    <t>3. UI mode for execution - npx playwright test &lt;spec file name&gt; --ui</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. Insurance sandbox html - </t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Test cases and scenarios</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     Data validation rules</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     </t>
+  </si>
+  <si>
+    <t xml:space="preserve">     In playwright, create a test for happy path of customer registration - sanitytest</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     Create a test for search for a non existant policy and it should say No policy found in sanitytest</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   </t>
+  </si>
+  <si>
+    <t xml:space="preserve">-Tip - Record the tests using npx playwright codegen &lt;htmlfilename&gt; </t>
+  </si>
+  <si>
+    <t xml:space="preserve">      copy the recorded script and paste in your spec.ts file </t>
+  </si>
+  <si>
+    <t xml:space="preserve">      add await expect to pass or fail the test</t>
+  </si>
+  <si>
+    <t>Framework structure-5 marks</t>
+  </si>
+  <si>
+    <t>SmokeTest-orangehome</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SanityTest -Login </t>
+  </si>
+  <si>
+    <t>Participant name</t>
+  </si>
+  <si>
+    <t>Validation - await expect</t>
+  </si>
+  <si>
+    <t>Total %</t>
+  </si>
+  <si>
+    <t>Mid assessment - 25 marks</t>
+  </si>
+  <si>
+    <t>Reusable modules &amp; Negative tc</t>
+  </si>
+  <si>
+    <t>sampledata</t>
+  </si>
+  <si>
+    <t>how to put the registration function as a reusable function in a module?</t>
+  </si>
+  <si>
+    <t>test (fn,ln,dob,email,phone,address) - successful</t>
+  </si>
+  <si>
+    <t>All ok</t>
+  </si>
+  <si>
+    <t>Any empty</t>
+  </si>
+  <si>
+    <t>Expect</t>
+  </si>
+  <si>
+    <t>Successful</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test ('',ln,dob,email,phone,address) - all fields are mandatory </t>
+  </si>
+  <si>
+    <t>unsuccessful</t>
+  </si>
+  <si>
+    <t>export function registerCustomer(fn :string, ln:string,dob :string,email:string,phone:number,add:string) {</t>
+  </si>
+  <si>
+    <t>}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fill the form </t>
+  </si>
+  <si>
+    <t>Typescript</t>
+  </si>
+  <si>
+    <t>tests</t>
+  </si>
+  <si>
+    <t>Sanitytests</t>
+  </si>
+  <si>
+    <t>utils</t>
+  </si>
+  <si>
+    <t>reg.spec.ts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     fillregform.ts</t>
+  </si>
+  <si>
+    <t>../../utils/fillregform.ts</t>
+  </si>
+  <si>
+    <t>VPN Issue.</t>
+  </si>
+  <si>
+    <t>Not responding (Restarted) will showcase 08/Sep - reported some emergency</t>
+  </si>
+  <si>
+    <t>test('Check position of Register customer button @ui', async ({ page }) =&gt; {</t>
+  </si>
+  <si>
+    <t>test ('Check the style @ui of the Register customer button ', async ({ page }) =&gt; {</t>
+  </si>
+  <si>
+    <t>test ('Check if the label for First Name input box @ui is First Name *', async ({ page }) =&gt; {</t>
+  </si>
+  <si>
+    <t>test('Check background colour of the Register customer @ui button to be dark blue ', async ({ page }) =&gt; {</t>
+  </si>
+  <si>
+    <t>#163a5f</t>
+  </si>
+  <si>
+    <t>not present</t>
+  </si>
+  <si>
+    <t>Status as on 9 Sep</t>
+  </si>
+  <si>
+    <t>Done during evaluation</t>
+  </si>
+  <si>
+    <t>Will showcase 10/Sep</t>
+  </si>
+  <si>
+    <t>Insurance</t>
+  </si>
+  <si>
+    <t>Tables</t>
+  </si>
+  <si>
+    <t>Customers</t>
+  </si>
+  <si>
+    <t>Custid</t>
+  </si>
+  <si>
+    <t>custname</t>
+  </si>
+  <si>
+    <t>Add 1</t>
+  </si>
+  <si>
+    <t>Add 2</t>
+  </si>
+  <si>
+    <t>City</t>
+  </si>
+  <si>
+    <t>State</t>
+  </si>
+  <si>
+    <t>Pincode</t>
+  </si>
+  <si>
+    <t>email</t>
+  </si>
+  <si>
+    <t>phone</t>
+  </si>
+  <si>
+    <t>create database - db lead</t>
+  </si>
+  <si>
+    <t>c001</t>
+  </si>
+  <si>
+    <t>Bala</t>
+  </si>
+  <si>
+    <t>7,abcd</t>
+  </si>
+  <si>
+    <t>Chennai</t>
+  </si>
+  <si>
+    <t>TN</t>
+  </si>
+  <si>
+    <t>abc@gmail.com</t>
+  </si>
+  <si>
+    <t>Registration screen</t>
+  </si>
+  <si>
+    <t>https://insonline.com</t>
+  </si>
+  <si>
+    <t>Sign up</t>
+  </si>
+  <si>
+    <t>Sign in</t>
+  </si>
+  <si>
+    <t>password</t>
+  </si>
+  <si>
+    <t>confirm password</t>
+  </si>
+  <si>
+    <t>Personal detail</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Name </t>
+  </si>
+  <si>
+    <t>Add1</t>
+  </si>
+  <si>
+    <t>Add2</t>
+  </si>
+  <si>
+    <t>email id</t>
+  </si>
+  <si>
+    <t>Policies</t>
+  </si>
+  <si>
+    <t>Status of policy</t>
+  </si>
+  <si>
+    <t>Admin modules</t>
+  </si>
+  <si>
+    <t>https://insonline.com/admin</t>
+  </si>
+  <si>
+    <t>create policy</t>
+  </si>
+  <si>
+    <t>Normal logged in user clicks policies</t>
+  </si>
+  <si>
+    <t>Transactions/My policy</t>
+  </si>
+  <si>
+    <t>Policy name</t>
+  </si>
+  <si>
+    <t>Applicable to ages</t>
+  </si>
+  <si>
+    <t>Term</t>
+  </si>
+  <si>
+    <t>Turnover</t>
+  </si>
+  <si>
+    <t>Bhima nivesh</t>
+  </si>
+  <si>
+    <t>Ages 15 - 30</t>
+  </si>
+  <si>
+    <t>Policies table</t>
+  </si>
+  <si>
+    <t>Buy</t>
+  </si>
+  <si>
+    <t>Premium</t>
+  </si>
+  <si>
+    <t>Update policy</t>
+  </si>
+  <si>
+    <t>Delete policy</t>
+  </si>
+  <si>
+    <t>Edit - policy</t>
+  </si>
+  <si>
+    <t>Creation - Data Definition language</t>
+  </si>
+  <si>
+    <t>Create database insonline</t>
+  </si>
+  <si>
+    <t>create table customer (custid char(4), custname char(20),dob date , email char(25), …)</t>
+  </si>
+  <si>
+    <t>Data Manipulation language</t>
+  </si>
+  <si>
+    <t>Update,delete</t>
+  </si>
+  <si>
+    <t>DDL, DML, DCL</t>
+  </si>
+  <si>
+    <t>Grant connect to Admin identified by admin123</t>
+  </si>
+  <si>
+    <t>Admin - DCL</t>
+  </si>
+  <si>
+    <t>Authorization</t>
+  </si>
+  <si>
+    <t>Primary key</t>
+  </si>
+  <si>
+    <t>Master</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Users </t>
+  </si>
+  <si>
+    <t>username</t>
+  </si>
+  <si>
+    <t>create</t>
+  </si>
+  <si>
+    <t>update</t>
+  </si>
+  <si>
+    <t>delete</t>
+  </si>
+  <si>
+    <t>edit</t>
+  </si>
+  <si>
+    <t>Insert into users values("Admin1","admin123","Y","Y","Y","Y")</t>
+  </si>
+  <si>
+    <t>Insert into users values("Admin","admin123","Y","Y","N","y")</t>
+  </si>
+  <si>
+    <t>Customer</t>
+  </si>
+  <si>
+    <t>policy1</t>
+  </si>
+  <si>
+    <t>policy2</t>
+  </si>
+  <si>
+    <t>policy3</t>
+  </si>
+  <si>
+    <t>One to many relationship</t>
+  </si>
+  <si>
+    <t>c002</t>
+  </si>
+  <si>
+    <t>ABCD</t>
+  </si>
+  <si>
+    <t>d03</t>
+  </si>
+  <si>
+    <t>1CR</t>
+  </si>
+  <si>
+    <t>List all the orders sorted by customers</t>
+  </si>
+  <si>
+    <t>SELECT orders.orderid, orders.orderdate, orders.customerid,customers.customername FROM Orders , customers where orders.customerid = customers.customerid order by orders.customerid</t>
+  </si>
+  <si>
+    <t>SELECT o.orderid, o.orderdate, o.customerid,c.customername FROM Orders as o , customers as c where o.customerid = c.customerid order by o.customerid</t>
+  </si>
+  <si>
+    <t>aliases</t>
+  </si>
+  <si>
+    <t>SELECT orderid,productid,quantity FROM OrderDetails;</t>
+  </si>
+  <si>
+    <t>orderdetails</t>
+  </si>
+  <si>
+    <t>OrderID</t>
+  </si>
+  <si>
+    <t>CustomerID</t>
+  </si>
+  <si>
+    <t>EmployeeID</t>
+  </si>
+  <si>
+    <t>OrderDate</t>
+  </si>
+  <si>
+    <t>orders table</t>
+  </si>
+  <si>
+    <t>select orderid,productid,quantity, customerid,customername, employeeid from orderdetails,orders,customers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">select od.orderid,od.productid,od.quantity, o.customerid,c.customername, o.employeeid from orderdetails as od,orders as o ,customers as c </t>
+  </si>
+  <si>
+    <t>where od.orderid= orders.orderid</t>
+  </si>
+  <si>
+    <t xml:space="preserve">and </t>
+  </si>
+  <si>
+    <t>o.customerid=c.customerid</t>
+  </si>
+  <si>
+    <t>o.customerid=c.customerid order by o.customerid</t>
+  </si>
+  <si>
+    <t>select od.orderid,od.productid,od.quantity, p.price, o.customerid,c.customername, o.employeeid ,e.firstname from orderdetails as od,orders as o ,customers as c ,products as p,employees as e</t>
+  </si>
+  <si>
+    <t>where od.orderid= o.orderid and o.employeeid = e.employeeid and od.productid =p.productid</t>
+  </si>
+  <si>
+    <t>select od.orderid,od.productid,od.quantity, p.price, od.quantity * p.price as "Total" , o.customerid,c.customername, o.employeeid ,e.firstname as "agentname" from orderdetails as od,orders as o ,customers as c ,products as p,employees as e</t>
+  </si>
+  <si>
+    <t>customerwise order detail along with order total</t>
+  </si>
+  <si>
+    <t>SELECT p.productname,p.categoryid,c.categoryname , c.description from</t>
+  </si>
+  <si>
+    <t xml:space="preserve">products as p, categories as c </t>
+  </si>
+  <si>
+    <t>where</t>
+  </si>
+  <si>
+    <t>p.categoryid=c.categoryid</t>
+  </si>
+  <si>
+    <t>for product name</t>
+  </si>
+  <si>
+    <t>Working query - shopping cart</t>
+  </si>
+  <si>
+    <t>o.customerid=c.customerid and o.customerid=7</t>
+  </si>
+  <si>
+    <t>Indexes</t>
+  </si>
+  <si>
+    <t>Harry</t>
+  </si>
+  <si>
+    <t>c003</t>
+  </si>
+  <si>
+    <t>Ria</t>
+  </si>
+  <si>
+    <t>c004</t>
+  </si>
+  <si>
+    <t>Helen</t>
+  </si>
+  <si>
+    <t>customername</t>
+  </si>
+  <si>
+    <t>select customername from customers</t>
+  </si>
+  <si>
+    <t>list customers by name</t>
+  </si>
+  <si>
+    <t>Index</t>
+  </si>
+  <si>
+    <t>Create index custnameindex as (select customername from customers)</t>
+  </si>
+  <si>
+    <t>c005</t>
+  </si>
+  <si>
+    <t>Aman</t>
+  </si>
+  <si>
+    <t>c006</t>
+  </si>
+  <si>
+    <t>Balu</t>
+  </si>
+  <si>
+    <t>Reindex</t>
+  </si>
+  <si>
+    <t>Sales</t>
+  </si>
+  <si>
+    <t>E</t>
+  </si>
+  <si>
+    <t>W</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>S</t>
+  </si>
+  <si>
+    <t>Zone</t>
+  </si>
+  <si>
+    <t>O1</t>
+  </si>
+  <si>
+    <t>O2</t>
+  </si>
+  <si>
+    <t>ZONE</t>
+  </si>
+  <si>
+    <t>Branch</t>
+  </si>
+  <si>
+    <t>Agentcode</t>
+  </si>
+  <si>
+    <t>A01</t>
+  </si>
+  <si>
+    <t>A03</t>
+  </si>
+  <si>
+    <t>A21</t>
+  </si>
+  <si>
+    <t>A04</t>
+  </si>
+  <si>
+    <t>declarion of vars</t>
+  </si>
+  <si>
+    <t>assigning value to vars</t>
+  </si>
+  <si>
+    <t>using vars in loops</t>
+  </si>
+  <si>
+    <t>boundary</t>
+  </si>
+  <si>
+    <t>conditional stmts</t>
+  </si>
+  <si>
+    <t>x = 5</t>
+  </si>
+  <si>
+    <t>number x</t>
+  </si>
+  <si>
+    <t>for I=0;I &lt; x ;I ++</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   if (I %2) ===0 then print even</t>
+  </si>
+  <si>
+    <t>else print odd</t>
+  </si>
+  <si>
+    <t>end of for</t>
+  </si>
+  <si>
+    <t>no print</t>
+  </si>
+  <si>
+    <t xml:space="preserve">expected </t>
+  </si>
+  <si>
+    <t>if x</t>
+  </si>
+  <si>
+    <t xml:space="preserve">if x </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>print even and odd numbers</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="30" x14ac:knownFonts="1">
+  <fonts count="38" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -5834,8 +6755,62 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF424242"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFCE9178"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF242424"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Verdana"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -5884,8 +6859,26 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="6">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -5960,11 +6953,49 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -6073,8 +7104,57 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="31" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="37" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="11" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -6385,6 +7465,26 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="3">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{21224A79-E9C3-4F0C-ABF2-35BCC58FA90A}">
+  <we:reference id="wa200005669" version="2.0.0.0" store="en-US" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="wa200005669" version="2.0.0.0" store="wa200005669" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties/>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0AD45E7A-FE4A-44C4-B18D-FF22DFDF16A9}">
   <dimension ref="A4:O106"/>
@@ -6542,6 +7642,158 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{47B9EBFF-FAB7-40C2-8100-85EAFB904205}">
+  <dimension ref="B3:M100"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="3" spans="4:13" x14ac:dyDescent="0.25">
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+      <c r="G3" s="48">
+        <v>2</v>
+      </c>
+      <c r="H3">
+        <v>3</v>
+      </c>
+      <c r="I3" s="48">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="4:13" x14ac:dyDescent="0.25">
+      <c r="D4" t="s">
+        <v>570</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="F4">
+        <v>2</v>
+      </c>
+      <c r="G4">
+        <v>3</v>
+      </c>
+      <c r="H4">
+        <v>4</v>
+      </c>
+      <c r="I4">
+        <v>5</v>
+      </c>
+      <c r="L4" t="s">
+        <v>579</v>
+      </c>
+    </row>
+    <row r="6" spans="4:13" x14ac:dyDescent="0.25">
+      <c r="D6" t="s">
+        <v>571</v>
+      </c>
+      <c r="L6" t="s">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="7" spans="4:13" x14ac:dyDescent="0.25">
+      <c r="L7" t="s">
+        <v>576</v>
+      </c>
+    </row>
+    <row r="8" spans="4:13" x14ac:dyDescent="0.25">
+      <c r="E8" t="s">
+        <v>572</v>
+      </c>
+      <c r="I8" t="s">
+        <v>573</v>
+      </c>
+      <c r="L8" t="s">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="9" spans="4:13" x14ac:dyDescent="0.25">
+      <c r="I9" t="s">
+        <v>574</v>
+      </c>
+    </row>
+    <row r="10" spans="4:13" x14ac:dyDescent="0.25">
+      <c r="I10" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="12" spans="4:13" x14ac:dyDescent="0.25">
+      <c r="H12" t="s">
+        <v>580</v>
+      </c>
+      <c r="K12" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="13" spans="4:13" x14ac:dyDescent="0.25">
+      <c r="H13" t="s">
+        <v>586</v>
+      </c>
+      <c r="K13" t="s">
+        <v>581</v>
+      </c>
+      <c r="L13" t="s">
+        <v>582</v>
+      </c>
+      <c r="M13" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="14" spans="4:13" x14ac:dyDescent="0.25">
+      <c r="K14" t="s">
+        <v>183</v>
+      </c>
+      <c r="L14" t="s">
+        <v>583</v>
+      </c>
+      <c r="M14" t="s">
+        <v>585</v>
+      </c>
+    </row>
+    <row r="16" spans="4:13" x14ac:dyDescent="0.25">
+      <c r="K16" t="s">
+        <v>588</v>
+      </c>
+    </row>
+    <row r="100" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B100" t="s">
+        <v>569</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{913ED22E-69BE-48F7-94C8-6CAB8D4B66E4}">
+  <dimension ref="C99:C101"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="99" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C99" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="100" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C100" t="s">
+        <v>589</v>
+      </c>
+    </row>
+    <row r="101" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C101" t="s">
+        <v>590</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C7CD2AC4-7135-45AD-B278-1DBC17B0666E}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -6552,14 +7804,1068 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D90C64F2-34FE-4740-BA7F-B01B1E462906}">
-  <dimension ref="A1"/>
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:Q92"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="5" max="5" width="13.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="3:17" x14ac:dyDescent="0.25">
+      <c r="E1" t="s">
+        <v>611</v>
+      </c>
+    </row>
+    <row r="2" spans="3:17" x14ac:dyDescent="0.25">
+      <c r="D2" s="48" t="s">
+        <v>602</v>
+      </c>
+      <c r="E2" s="48" t="s">
+        <v>603</v>
+      </c>
+      <c r="F2" s="48" t="s">
+        <v>606</v>
+      </c>
+      <c r="G2" s="48" t="s">
+        <v>607</v>
+      </c>
+      <c r="H2" s="48" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="3" spans="3:17" x14ac:dyDescent="0.25">
+      <c r="C3" t="s">
+        <v>601</v>
+      </c>
+      <c r="D3" t="s">
+        <v>604</v>
+      </c>
+      <c r="E3" t="s">
+        <v>604</v>
+      </c>
+      <c r="F3" t="b">
+        <v>1</v>
+      </c>
+      <c r="G3" t="b">
+        <v>1</v>
+      </c>
+      <c r="H3" t="s">
+        <v>39</v>
+      </c>
+      <c r="I3" t="s">
+        <v>612</v>
+      </c>
+      <c r="J3" t="s">
+        <v>616</v>
+      </c>
+      <c r="O3" t="s">
+        <v>620</v>
+      </c>
+      <c r="P3" t="s">
+        <v>621</v>
+      </c>
+    </row>
+    <row r="4" spans="3:17" x14ac:dyDescent="0.25">
+      <c r="C4" t="s">
+        <v>608</v>
+      </c>
+      <c r="D4" t="s">
+        <v>604</v>
+      </c>
+      <c r="E4" t="s">
+        <v>609</v>
+      </c>
+      <c r="F4" t="b">
+        <v>0</v>
+      </c>
+      <c r="G4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H4" t="s">
+        <v>40</v>
+      </c>
+      <c r="I4" t="s">
+        <v>613</v>
+      </c>
+      <c r="K4" t="s">
+        <v>614</v>
+      </c>
+    </row>
+    <row r="5" spans="3:17" x14ac:dyDescent="0.25">
+      <c r="C5" t="s">
+        <v>610</v>
+      </c>
+      <c r="D5" t="s">
+        <v>609</v>
+      </c>
+      <c r="E5" t="s">
+        <v>609</v>
+      </c>
+      <c r="F5" t="b">
+        <v>0</v>
+      </c>
+      <c r="G5" t="b">
+        <v>1</v>
+      </c>
+      <c r="H5" t="s">
+        <v>40</v>
+      </c>
+      <c r="I5" t="s">
+        <v>613</v>
+      </c>
+      <c r="K5" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="6" spans="3:17" x14ac:dyDescent="0.25">
+      <c r="C6" t="s">
+        <v>622</v>
+      </c>
+      <c r="D6" t="s">
+        <v>623</v>
+      </c>
+      <c r="E6" t="s">
+        <v>604</v>
+      </c>
+      <c r="F6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="3:17" x14ac:dyDescent="0.25">
+      <c r="E12" t="s">
+        <v>619</v>
+      </c>
+      <c r="F12" t="s">
+        <v>617</v>
+      </c>
+      <c r="G12" t="s">
+        <v>618</v>
+      </c>
+      <c r="I12" t="s">
+        <v>605</v>
+      </c>
+    </row>
+    <row r="15" spans="3:17" x14ac:dyDescent="0.25">
+      <c r="J15" t="s">
+        <v>624</v>
+      </c>
+      <c r="K15" t="s">
+        <v>625</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>630</v>
+      </c>
+    </row>
+    <row r="16" spans="3:17" x14ac:dyDescent="0.25">
+      <c r="J16" t="s">
+        <v>627</v>
+      </c>
+      <c r="K16" t="s">
+        <v>628</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="J17" t="s">
+        <v>626</v>
+      </c>
+      <c r="K17" t="s">
+        <v>629</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="F18" t="s">
+        <v>631</v>
+      </c>
+      <c r="G18" t="s">
+        <v>607</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E19" t="s">
+        <v>629</v>
+      </c>
+      <c r="F19">
+        <v>120</v>
+      </c>
+      <c r="G19">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="H21" t="s">
+        <v>629</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D23" t="s">
+        <v>632</v>
+      </c>
+      <c r="E23" t="s">
+        <v>633</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>634</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>635</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>636</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>637</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>638</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>640</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>641</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>642</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>644</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>646</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>647</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>652</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>656</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>657</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>658</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>660</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>661</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>663</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>665</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>666</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>668</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>670</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>594</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>597</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>598</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>674</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>599</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>594</v>
+      </c>
+    </row>
+    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="79" spans="1:1" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="80" spans="1:1" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>597</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>598</v>
+      </c>
+    </row>
+    <row r="82" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>675</v>
+      </c>
+    </row>
+    <row r="83" spans="1:1" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="84" spans="1:1" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>677</v>
+      </c>
+    </row>
+    <row r="85" spans="1:1" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>678</v>
+      </c>
+    </row>
+    <row r="86" spans="1:1" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="87" spans="1:1" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>680</v>
+      </c>
+    </row>
+    <row r="88" spans="1:1" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>681</v>
+      </c>
+    </row>
+    <row r="89" spans="1:1" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="90" spans="1:1" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>683</v>
+      </c>
+    </row>
+    <row r="91" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>684</v>
+      </c>
+    </row>
+    <row r="92" spans="1:1" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>685</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A30:Q92" xr:uid="{D90C64F2-34FE-4740-BA7F-B01B1E462906}">
+    <filterColumn colId="0">
+      <customFilters>
+        <customFilter val="*BROKEN*"/>
+      </customFilters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91A716CE-CFD6-4ADE-9CE5-1AFF6EA62D47}">
+  <dimension ref="A1:H107"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="26" customWidth="1"/>
+    <col min="2" max="2" width="14.42578125" customWidth="1"/>
+    <col min="3" max="3" width="10.42578125" customWidth="1"/>
+    <col min="4" max="4" width="9" customWidth="1"/>
+    <col min="5" max="5" width="12.140625" customWidth="1"/>
+    <col min="6" max="6" width="11" customWidth="1"/>
+    <col min="8" max="8" width="37.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>691</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>692</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>693</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>695</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>696</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>697</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>698</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>701</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>703</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>704</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>706</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" s="51"/>
+      <c r="B22" s="51"/>
+      <c r="C22" s="52" t="s">
+        <v>713</v>
+      </c>
+      <c r="D22" s="51"/>
+      <c r="E22" s="51"/>
+      <c r="F22" s="51"/>
+      <c r="G22" s="51"/>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" s="51"/>
+      <c r="B23" s="51"/>
+      <c r="C23" s="51"/>
+      <c r="D23" s="51"/>
+      <c r="E23" s="51"/>
+      <c r="F23" s="51"/>
+      <c r="G23" s="51"/>
+    </row>
+    <row r="24" spans="1:8" s="58" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="56" t="s">
+        <v>710</v>
+      </c>
+      <c r="B24" s="56" t="s">
+        <v>707</v>
+      </c>
+      <c r="C24" s="56" t="s">
+        <v>708</v>
+      </c>
+      <c r="D24" s="56" t="s">
+        <v>709</v>
+      </c>
+      <c r="E24" s="56" t="s">
+        <v>714</v>
+      </c>
+      <c r="F24" s="56" t="s">
+        <v>711</v>
+      </c>
+      <c r="G24" s="56" t="s">
+        <v>712</v>
+      </c>
+      <c r="H24" s="57" t="s">
+        <v>742</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" s="62" customFormat="1" ht="12" x14ac:dyDescent="0.2">
+      <c r="A25" s="59" t="s">
+        <v>95</v>
+      </c>
+      <c r="B25" s="60">
+        <v>4</v>
+      </c>
+      <c r="C25" s="60">
+        <v>4</v>
+      </c>
+      <c r="D25" s="60">
+        <v>5</v>
+      </c>
+      <c r="E25" s="60">
+        <v>3</v>
+      </c>
+      <c r="F25" s="60">
+        <v>5</v>
+      </c>
+      <c r="G25" s="61">
+        <f>(SUM(B25:F25)/25)*100</f>
+        <v>84</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" s="62" customFormat="1" ht="12" x14ac:dyDescent="0.2">
+      <c r="A26" s="59" t="s">
+        <v>99</v>
+      </c>
+      <c r="B26" s="60">
+        <v>5</v>
+      </c>
+      <c r="C26" s="60">
+        <v>5</v>
+      </c>
+      <c r="D26" s="60">
+        <v>4</v>
+      </c>
+      <c r="E26" s="60">
+        <v>2</v>
+      </c>
+      <c r="F26" s="60">
+        <v>5</v>
+      </c>
+      <c r="G26" s="61">
+        <f>(SUM(B26:F26)/25)*100</f>
+        <v>84</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" s="62" customFormat="1" ht="12" x14ac:dyDescent="0.2">
+      <c r="A27" s="63" t="s">
+        <v>715</v>
+      </c>
+      <c r="B27" s="60">
+        <v>4</v>
+      </c>
+      <c r="C27" s="60">
+        <v>3</v>
+      </c>
+      <c r="D27" s="60">
+        <v>5</v>
+      </c>
+      <c r="E27" s="60">
+        <v>3</v>
+      </c>
+      <c r="F27" s="60">
+        <v>5</v>
+      </c>
+      <c r="G27" s="61">
+        <f>(SUM(B27:F27)/25)*100</f>
+        <v>80</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" s="62" customFormat="1" ht="12" x14ac:dyDescent="0.2">
+      <c r="A28" s="59" t="s">
+        <v>94</v>
+      </c>
+      <c r="B28" s="60">
+        <v>3</v>
+      </c>
+      <c r="C28" s="60">
+        <v>0</v>
+      </c>
+      <c r="D28" s="60">
+        <v>3</v>
+      </c>
+      <c r="E28" s="60">
+        <v>2</v>
+      </c>
+      <c r="F28" s="60">
+        <v>4</v>
+      </c>
+      <c r="G28" s="61">
+        <f>(SUM(B28:F28)/25)*100</f>
+        <v>48</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" s="62" customFormat="1" ht="12" x14ac:dyDescent="0.2">
+      <c r="A29" s="59" t="s">
+        <v>96</v>
+      </c>
+      <c r="B29" s="65" t="s">
+        <v>735</v>
+      </c>
+      <c r="C29" s="60"/>
+      <c r="D29" s="60"/>
+      <c r="E29" s="60"/>
+      <c r="F29" s="60"/>
+      <c r="G29" s="61"/>
+      <c r="H29" s="62" t="s">
+        <v>741</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" s="62" customFormat="1" ht="12" x14ac:dyDescent="0.2">
+      <c r="A30" s="59" t="s">
+        <v>97</v>
+      </c>
+      <c r="B30" s="60">
+        <v>4</v>
+      </c>
+      <c r="C30" s="60">
+        <v>3</v>
+      </c>
+      <c r="D30" s="60">
+        <v>3</v>
+      </c>
+      <c r="E30" s="60">
+        <v>3</v>
+      </c>
+      <c r="F30" s="60">
+        <v>3</v>
+      </c>
+      <c r="G30" s="61">
+        <f>(SUM(B30:F30)/25)*100</f>
+        <v>64</v>
+      </c>
+      <c r="H30" s="62" t="s">
+        <v>743</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" s="62" customFormat="1" ht="12" x14ac:dyDescent="0.2">
+      <c r="A31" s="59" t="s">
+        <v>100</v>
+      </c>
+      <c r="B31" s="60" t="s">
+        <v>734</v>
+      </c>
+      <c r="C31" s="60"/>
+      <c r="D31" s="60"/>
+      <c r="E31" s="60"/>
+      <c r="F31" s="60"/>
+      <c r="G31" s="61"/>
+    </row>
+    <row r="32" spans="1:8" s="62" customFormat="1" ht="12" x14ac:dyDescent="0.2">
+      <c r="A32" s="59" t="s">
+        <v>101</v>
+      </c>
+      <c r="B32" s="60" t="s">
+        <v>744</v>
+      </c>
+      <c r="C32" s="60"/>
+      <c r="D32" s="60"/>
+      <c r="E32" s="60"/>
+      <c r="F32" s="60"/>
+      <c r="G32" s="61"/>
+    </row>
+    <row r="33" spans="1:7" s="62" customFormat="1" ht="12" x14ac:dyDescent="0.2">
+      <c r="A33" s="64" t="s">
+        <v>98</v>
+      </c>
+      <c r="B33" s="60" t="s">
+        <v>744</v>
+      </c>
+      <c r="C33" s="60"/>
+      <c r="D33" s="60"/>
+      <c r="E33" s="60"/>
+      <c r="F33" s="60"/>
+      <c r="G33" s="61"/>
+    </row>
+    <row r="34" spans="1:7" s="62" customFormat="1" ht="12" x14ac:dyDescent="0.2"/>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C51" t="s">
+        <v>716</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D53" t="s">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>718</v>
+      </c>
+      <c r="B54" t="s">
+        <v>717</v>
+      </c>
+      <c r="D54" t="s">
+        <v>721</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>719</v>
+      </c>
+      <c r="B55" t="s">
+        <v>722</v>
+      </c>
+      <c r="D55" t="s">
+        <v>723</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C59" t="s">
+        <v>724</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C61" t="s">
+        <v>726</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C64" t="s">
+        <v>725</v>
+      </c>
+    </row>
+    <row r="76" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C76" t="s">
+        <v>727</v>
+      </c>
+      <c r="D76" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="77" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="E77" t="s">
+        <v>729</v>
+      </c>
+      <c r="F77" s="2" t="s">
+        <v>731</v>
+      </c>
+    </row>
+    <row r="85" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D85" t="s">
+        <v>730</v>
+      </c>
+    </row>
+    <row r="86" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D86" t="s">
+        <v>732</v>
+      </c>
+      <c r="E86" t="s">
+        <v>733</v>
+      </c>
+    </row>
+    <row r="99" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C99" t="s">
+        <v>688</v>
+      </c>
+      <c r="D99" t="s">
+        <v>689</v>
+      </c>
+      <c r="E99" t="s">
+        <v>690</v>
+      </c>
+    </row>
+    <row r="100" spans="3:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="C100" s="7" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="101" spans="3:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="C101" s="7" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="102" spans="3:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="C102" s="7" t="s">
+        <v>686</v>
+      </c>
+    </row>
+    <row r="103" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C103" s="50" t="s">
+        <v>687</v>
+      </c>
+    </row>
+    <row r="104" spans="3:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="C104" s="7" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="105" spans="3:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="C105" s="7" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="106" spans="3:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="C106" s="7" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="107" spans="3:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="C107" s="7" t="s">
+        <v>102</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A24:G33" xr:uid="{91A716CE-CFD6-4ADE-9CE5-1AFF6EA62D47}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A25:G33">
+      <sortCondition descending="1" ref="G24:G33"/>
+    </sortState>
+  </autoFilter>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22A90608-B396-45C9-9755-E66FC11DDD67}">
+  <dimension ref="A1:D17"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="53"/>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="54"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="54"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="53" t="s">
+        <v>736</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="53" t="s">
+        <v>737</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="53" t="s">
+        <v>738</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="53" t="s">
+        <v>739</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="54"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="53"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="54"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="53"/>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="54"/>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="53"/>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="54"/>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="53"/>
+      <c r="D15" s="55" t="s">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="54"/>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" s="53"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B7E443E-A784-46FE-8849-1FF7656C16F4}">
   <dimension ref="B5:L119"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -7017,7 +9323,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{236DA920-215A-459D-AE62-6D5998601A03}">
   <dimension ref="A1:C484"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -9473,7 +11779,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F59EF5E-04B9-4C14-BD21-02325F9D115C}">
   <dimension ref="A1:N109"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -9740,16 +12046,925 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0EDDD263-AF87-495D-97B2-8E957BF524B9}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:S165"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="2" max="2" width="13.28515625" customWidth="1"/>
+    <col min="11" max="11" width="15.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="32" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A2" s="26" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A3" s="26" t="s">
+        <v>425</v>
+      </c>
+      <c r="K3" t="s">
+        <v>745</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A4" s="26" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A5" s="26" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A6" s="26" t="s">
+        <v>428</v>
+      </c>
+      <c r="K6" s="44" t="s">
+        <v>746</v>
+      </c>
+      <c r="N6" t="s">
+        <v>757</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A7" s="26" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A8" s="26" t="s">
+        <v>430</v>
+      </c>
+      <c r="J8" t="s">
+        <v>804</v>
+      </c>
+      <c r="K8" s="44" t="s">
+        <v>747</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A9" s="26" t="s">
+        <v>431</v>
+      </c>
+      <c r="K9" s="44" t="s">
+        <v>748</v>
+      </c>
+      <c r="L9" s="44" t="s">
+        <v>749</v>
+      </c>
+      <c r="M9" s="44" t="s">
+        <v>750</v>
+      </c>
+      <c r="N9" s="44" t="s">
+        <v>751</v>
+      </c>
+      <c r="O9" s="44" t="s">
+        <v>752</v>
+      </c>
+      <c r="P9" s="44" t="s">
+        <v>753</v>
+      </c>
+      <c r="Q9" s="44" t="s">
+        <v>754</v>
+      </c>
+      <c r="R9" s="44" t="s">
+        <v>755</v>
+      </c>
+      <c r="S9" s="44" t="s">
+        <v>756</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A10" s="26" t="s">
+        <v>432</v>
+      </c>
+      <c r="J10" t="s">
+        <v>803</v>
+      </c>
+      <c r="K10" s="44" t="s">
+        <v>758</v>
+      </c>
+      <c r="L10" t="s">
+        <v>759</v>
+      </c>
+      <c r="M10" t="s">
+        <v>760</v>
+      </c>
+      <c r="N10">
+        <v>323</v>
+      </c>
+      <c r="O10" t="s">
+        <v>761</v>
+      </c>
+      <c r="P10" t="s">
+        <v>762</v>
+      </c>
+      <c r="Q10">
+        <v>600093</v>
+      </c>
+      <c r="R10" s="66" t="s">
+        <v>763</v>
+      </c>
+      <c r="S10">
+        <v>52729829</v>
+      </c>
+    </row>
+    <row r="11" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A11" s="26" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="12" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A12" s="26" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="13" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A13" s="26" t="s">
+        <v>435</v>
+      </c>
+      <c r="O13" t="s">
+        <v>764</v>
+      </c>
+    </row>
+    <row r="14" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A14" s="26" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="15" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A15" s="26" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="16" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A16" s="26" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A17" s="26" t="s">
+        <v>439</v>
+      </c>
+      <c r="K17" s="66" t="s">
+        <v>765</v>
+      </c>
+      <c r="O17" t="s">
+        <v>755</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A18" s="32" t="s">
+        <v>419</v>
+      </c>
+      <c r="O18" t="s">
+        <v>768</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A19" s="32" t="s">
+        <v>440</v>
+      </c>
+      <c r="K19" t="s">
+        <v>766</v>
+      </c>
+      <c r="L19" t="s">
+        <v>29</v>
+      </c>
+      <c r="O19" t="s">
+        <v>769</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="K20" t="s">
+        <v>767</v>
+      </c>
+      <c r="L20" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="O21" t="s">
+        <v>770</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="O22" t="s">
+        <v>771</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="O23" t="s">
+        <v>772</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="G24" s="44" t="s">
+        <v>306</v>
+      </c>
+      <c r="O24" t="s">
+        <v>773</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="O25" t="s">
+        <v>752</v>
+      </c>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="E26" t="s">
+        <v>774</v>
+      </c>
+      <c r="O26" t="s">
+        <v>753</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="E27" t="s">
+        <v>25</v>
+      </c>
+      <c r="O27" t="s">
+        <v>754</v>
+      </c>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="F28" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="L29" t="s">
+        <v>799</v>
+      </c>
+      <c r="O29" t="s">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="K31" t="s">
+        <v>794</v>
+      </c>
+      <c r="O31" t="s">
+        <v>795</v>
+      </c>
+    </row>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="E32" t="s">
+        <v>775</v>
+      </c>
+      <c r="O32" t="s">
+        <v>796</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="E33" t="s">
+        <v>776</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="E34" t="s">
+        <v>781</v>
+      </c>
+      <c r="K34" t="s">
+        <v>798</v>
+      </c>
+      <c r="L34" t="s">
+        <v>797</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="K35" t="s">
+        <v>777</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="I37" s="66" t="s">
+        <v>778</v>
+      </c>
+      <c r="L37" t="s">
+        <v>802</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="J39" t="s">
+        <v>779</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="J40" t="s">
+        <v>791</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>780</v>
+      </c>
+      <c r="J41" t="s">
+        <v>792</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="J42" t="s">
+        <v>793</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="C43" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>748</v>
+      </c>
+      <c r="B44" s="44" t="s">
+        <v>782</v>
+      </c>
+      <c r="C44" s="44" t="s">
+        <v>783</v>
+      </c>
+      <c r="D44" s="44" t="s">
+        <v>784</v>
+      </c>
+      <c r="E44" s="44" t="s">
+        <v>785</v>
+      </c>
+      <c r="F44" s="44" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>758</v>
+      </c>
+      <c r="B45" t="s">
+        <v>786</v>
+      </c>
+      <c r="C45" t="s">
+        <v>787</v>
+      </c>
+      <c r="D45">
+        <v>3</v>
+      </c>
+      <c r="E45">
+        <v>1000000</v>
+      </c>
+      <c r="F45">
+        <v>10000</v>
+      </c>
+      <c r="G45" t="s">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>818</v>
+      </c>
+      <c r="B46" t="s">
+        <v>819</v>
+      </c>
+      <c r="C46" t="s">
+        <v>820</v>
+      </c>
+      <c r="D46">
+        <v>20</v>
+      </c>
+      <c r="E46" t="s">
+        <v>821</v>
+      </c>
+      <c r="F46">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="J48" t="s">
+        <v>801</v>
+      </c>
+    </row>
+    <row r="49" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="J49" s="44" t="s">
+        <v>805</v>
+      </c>
+      <c r="K49" t="s">
+        <v>806</v>
+      </c>
+      <c r="L49" t="s">
+        <v>768</v>
+      </c>
+      <c r="M49" t="s">
+        <v>807</v>
+      </c>
+      <c r="N49" t="s">
+        <v>808</v>
+      </c>
+      <c r="O49" t="s">
+        <v>809</v>
+      </c>
+      <c r="P49" t="s">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="50" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="J50" t="s">
+        <v>812</v>
+      </c>
+    </row>
+    <row r="51" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="J51" t="s">
+        <v>811</v>
+      </c>
+    </row>
+    <row r="54" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="J54" t="s">
+        <v>817</v>
+      </c>
+    </row>
+    <row r="55" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G55" t="s">
+        <v>813</v>
+      </c>
+      <c r="H55" t="s">
+        <v>814</v>
+      </c>
+    </row>
+    <row r="56" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="H56" t="s">
+        <v>815</v>
+      </c>
+    </row>
+    <row r="57" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="H57" t="s">
+        <v>816</v>
+      </c>
+    </row>
+    <row r="70" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="D70" t="s">
+        <v>822</v>
+      </c>
+      <c r="H70" t="s">
+        <v>823</v>
+      </c>
+    </row>
+    <row r="71" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="G71" t="s">
+        <v>825</v>
+      </c>
+      <c r="H71" t="s">
+        <v>824</v>
+      </c>
+    </row>
+    <row r="78" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B78" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="80" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B80" t="s">
+        <v>826</v>
+      </c>
+      <c r="K80" t="s">
+        <v>833</v>
+      </c>
+    </row>
+    <row r="81" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B81" t="s">
+        <v>832</v>
+      </c>
+    </row>
+    <row r="82" spans="2:11" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B82" s="67" t="s">
+        <v>828</v>
+      </c>
+      <c r="C82" s="68" t="s">
+        <v>829</v>
+      </c>
+      <c r="D82" s="68" t="s">
+        <v>830</v>
+      </c>
+      <c r="E82" s="68" t="s">
+        <v>831</v>
+      </c>
+      <c r="F82" s="69"/>
+    </row>
+    <row r="83" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="K83" t="s">
+        <v>834</v>
+      </c>
+    </row>
+    <row r="84" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="K84" t="s">
+        <v>835</v>
+      </c>
+    </row>
+    <row r="85" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="K85" t="s">
+        <v>836</v>
+      </c>
+    </row>
+    <row r="86" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="K86" t="s">
+        <v>837</v>
+      </c>
+    </row>
+    <row r="89" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="K89" t="s">
+        <v>839</v>
+      </c>
+    </row>
+    <row r="90" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="K90" t="s">
+        <v>840</v>
+      </c>
+    </row>
+    <row r="91" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="K91" t="s">
+        <v>836</v>
+      </c>
+    </row>
+    <row r="92" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="K92" t="s">
+        <v>838</v>
+      </c>
+    </row>
+    <row r="94" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="K94" s="44" t="s">
+        <v>848</v>
+      </c>
+    </row>
+    <row r="95" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="K95" t="s">
+        <v>841</v>
+      </c>
+    </row>
+    <row r="96" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="K96" t="s">
+        <v>840</v>
+      </c>
+    </row>
+    <row r="97" spans="6:19" x14ac:dyDescent="0.25">
+      <c r="K97" t="s">
+        <v>836</v>
+      </c>
+    </row>
+    <row r="98" spans="6:19" x14ac:dyDescent="0.25">
+      <c r="K98" t="s">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="100" spans="6:19" x14ac:dyDescent="0.25">
+      <c r="K100" t="s">
+        <v>842</v>
+      </c>
+    </row>
+    <row r="102" spans="6:19" x14ac:dyDescent="0.25">
+      <c r="I102" t="s">
+        <v>847</v>
+      </c>
+      <c r="K102" t="s">
+        <v>843</v>
+      </c>
+    </row>
+    <row r="103" spans="6:19" x14ac:dyDescent="0.25">
+      <c r="K103" t="s">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="104" spans="6:19" x14ac:dyDescent="0.25">
+      <c r="K104" t="s">
+        <v>845</v>
+      </c>
+    </row>
+    <row r="105" spans="6:19" x14ac:dyDescent="0.25">
+      <c r="K105" t="s">
+        <v>846</v>
+      </c>
+    </row>
+    <row r="109" spans="6:19" x14ac:dyDescent="0.25">
+      <c r="R109" t="s">
+        <v>857</v>
+      </c>
+    </row>
+    <row r="110" spans="6:19" x14ac:dyDescent="0.25">
+      <c r="F110" t="s">
+        <v>860</v>
+      </c>
+    </row>
+    <row r="111" spans="6:19" x14ac:dyDescent="0.25">
+      <c r="F111" s="44" t="s">
+        <v>865</v>
+      </c>
+      <c r="M111" t="s">
+        <v>850</v>
+      </c>
+    </row>
+    <row r="112" spans="6:19" x14ac:dyDescent="0.25">
+      <c r="I112" t="s">
+        <v>859</v>
+      </c>
+      <c r="S112" t="s">
+        <v>858</v>
+      </c>
+    </row>
+    <row r="113" spans="8:19" x14ac:dyDescent="0.25">
+      <c r="H113">
+        <v>1</v>
+      </c>
+      <c r="I113" t="s">
+        <v>862</v>
+      </c>
+      <c r="M113" t="s">
+        <v>748</v>
+      </c>
+      <c r="N113" t="s">
+        <v>856</v>
+      </c>
+    </row>
+    <row r="114" spans="8:19" x14ac:dyDescent="0.25">
+      <c r="H114">
+        <v>2</v>
+      </c>
+      <c r="I114" t="s">
+        <v>759</v>
+      </c>
+      <c r="M114" t="s">
+        <v>758</v>
+      </c>
+      <c r="N114" t="s">
+        <v>759</v>
+      </c>
+      <c r="S114" t="s">
+        <v>759</v>
+      </c>
+    </row>
+    <row r="115" spans="8:19" x14ac:dyDescent="0.25">
+      <c r="H115">
+        <v>3</v>
+      </c>
+      <c r="I115" t="s">
+        <v>864</v>
+      </c>
+      <c r="M115" t="s">
+        <v>818</v>
+      </c>
+      <c r="N115" t="s">
+        <v>851</v>
+      </c>
+      <c r="S115" t="s">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="116" spans="8:19" x14ac:dyDescent="0.25">
+      <c r="H116">
+        <v>4</v>
+      </c>
+      <c r="I116" t="s">
+        <v>851</v>
+      </c>
+      <c r="M116" t="s">
+        <v>852</v>
+      </c>
+      <c r="N116" t="s">
+        <v>853</v>
+      </c>
+      <c r="S116" t="s">
+        <v>855</v>
+      </c>
+    </row>
+    <row r="117" spans="8:19" x14ac:dyDescent="0.25">
+      <c r="H117">
+        <v>5</v>
+      </c>
+      <c r="I117" t="s">
+        <v>855</v>
+      </c>
+      <c r="M117" t="s">
+        <v>854</v>
+      </c>
+      <c r="N117" t="s">
+        <v>855</v>
+      </c>
+      <c r="S117" t="s">
+        <v>853</v>
+      </c>
+    </row>
+    <row r="118" spans="8:19" x14ac:dyDescent="0.25">
+      <c r="H118">
+        <v>6</v>
+      </c>
+      <c r="I118" t="s">
+        <v>853</v>
+      </c>
+      <c r="M118" t="s">
+        <v>861</v>
+      </c>
+      <c r="N118" t="s">
+        <v>862</v>
+      </c>
+    </row>
+    <row r="119" spans="8:19" x14ac:dyDescent="0.25">
+      <c r="M119" t="s">
+        <v>863</v>
+      </c>
+      <c r="N119" t="s">
+        <v>864</v>
+      </c>
+    </row>
+    <row r="129" spans="11:14" x14ac:dyDescent="0.25">
+      <c r="L129" t="s">
+        <v>866</v>
+      </c>
+    </row>
+    <row r="130" spans="11:14" x14ac:dyDescent="0.25">
+      <c r="K130" t="s">
+        <v>871</v>
+      </c>
+    </row>
+    <row r="131" spans="11:14" x14ac:dyDescent="0.25">
+      <c r="K131" t="s">
+        <v>867</v>
+      </c>
+    </row>
+    <row r="132" spans="11:14" x14ac:dyDescent="0.25">
+      <c r="K132" t="s">
+        <v>868</v>
+      </c>
+    </row>
+    <row r="133" spans="11:14" x14ac:dyDescent="0.25">
+      <c r="K133" t="s">
+        <v>869</v>
+      </c>
+    </row>
+    <row r="134" spans="11:14" x14ac:dyDescent="0.25">
+      <c r="K134" t="s">
+        <v>870</v>
+      </c>
+    </row>
+    <row r="135" spans="11:14" x14ac:dyDescent="0.25">
+      <c r="K135" t="s">
+        <v>874</v>
+      </c>
+      <c r="L135" t="s">
+        <v>875</v>
+      </c>
+      <c r="M135" t="s">
+        <v>876</v>
+      </c>
+      <c r="N135" t="s">
+        <v>866</v>
+      </c>
+    </row>
+    <row r="136" spans="11:14" x14ac:dyDescent="0.25">
+      <c r="K136" t="s">
+        <v>867</v>
+      </c>
+      <c r="L136" t="s">
+        <v>872</v>
+      </c>
+      <c r="M136" t="s">
+        <v>877</v>
+      </c>
+      <c r="N136">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="137" spans="11:14" x14ac:dyDescent="0.25">
+      <c r="K137" t="s">
+        <v>868</v>
+      </c>
+      <c r="L137" t="s">
+        <v>872</v>
+      </c>
+      <c r="M137" t="s">
+        <v>878</v>
+      </c>
+      <c r="N137">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="138" spans="11:14" x14ac:dyDescent="0.25">
+      <c r="K138" t="s">
+        <v>869</v>
+      </c>
+      <c r="L138" t="s">
+        <v>873</v>
+      </c>
+      <c r="M138" t="s">
+        <v>879</v>
+      </c>
+      <c r="N138">
+        <v>300000</v>
+      </c>
+    </row>
+    <row r="139" spans="11:14" x14ac:dyDescent="0.25">
+      <c r="K139" t="s">
+        <v>867</v>
+      </c>
+      <c r="L139" t="s">
+        <v>873</v>
+      </c>
+      <c r="M139" t="s">
+        <v>880</v>
+      </c>
+      <c r="N139">
+        <v>7000004</v>
+      </c>
+    </row>
+    <row r="153" spans="11:18" x14ac:dyDescent="0.25">
+      <c r="K153" t="s">
+        <v>881</v>
+      </c>
+    </row>
+    <row r="154" spans="11:18" x14ac:dyDescent="0.25">
+      <c r="K154" t="s">
+        <v>882</v>
+      </c>
+    </row>
+    <row r="156" spans="11:18" x14ac:dyDescent="0.25">
+      <c r="K156" t="s">
+        <v>883</v>
+      </c>
+      <c r="M156" t="s">
+        <v>884</v>
+      </c>
+    </row>
+    <row r="158" spans="11:18" x14ac:dyDescent="0.25">
+      <c r="K158" t="s">
+        <v>885</v>
+      </c>
+      <c r="R158" t="s">
+        <v>893</v>
+      </c>
+    </row>
+    <row r="159" spans="11:18" x14ac:dyDescent="0.25">
+      <c r="M159" t="s">
+        <v>887</v>
+      </c>
+      <c r="Q159" t="s">
+        <v>894</v>
+      </c>
+      <c r="R159">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="160" spans="11:18" x14ac:dyDescent="0.25">
+      <c r="M160" t="s">
+        <v>886</v>
+      </c>
+      <c r="R160" t="s">
+        <v>892</v>
+      </c>
+    </row>
+    <row r="162" spans="13:18" x14ac:dyDescent="0.25">
+      <c r="M162" t="s">
+        <v>888</v>
+      </c>
+      <c r="Q162" t="s">
+        <v>895</v>
+      </c>
+      <c r="R162">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="163" spans="13:18" x14ac:dyDescent="0.25">
+      <c r="M163" t="s">
+        <v>889</v>
+      </c>
+      <c r="Q163" t="s">
+        <v>896</v>
+      </c>
+      <c r="R163" t="s">
+        <v>897</v>
+      </c>
+    </row>
+    <row r="164" spans="13:18" x14ac:dyDescent="0.25">
+      <c r="M164" t="s">
+        <v>890</v>
+      </c>
+    </row>
+    <row r="165" spans="13:18" x14ac:dyDescent="0.25">
+      <c r="M165" t="s">
+        <v>891</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="R10" r:id="rId1" xr:uid="{4115217A-C819-4494-9B37-F381CC96C3CA}"/>
+    <hyperlink ref="K17" r:id="rId2" xr:uid="{6D4AB588-5CC0-43E7-A22F-A70B6F621400}"/>
+    <hyperlink ref="I37" r:id="rId3" xr:uid="{1EC9773A-0875-4B11-B7C2-B63A7F8951DB}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9CB0199-FD5A-4BDA-AA2F-1DD098D56AA9}">
   <dimension ref="C2:C100"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -9783,156 +12998,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{47B9EBFF-FAB7-40C2-8100-85EAFB904205}">
-  <dimension ref="B3:M100"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="3" spans="4:13" x14ac:dyDescent="0.25">
-      <c r="E3">
-        <v>0</v>
-      </c>
-      <c r="F3">
-        <v>1</v>
-      </c>
-      <c r="G3" s="48">
-        <v>2</v>
-      </c>
-      <c r="H3">
-        <v>3</v>
-      </c>
-      <c r="I3" s="48">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="4:13" x14ac:dyDescent="0.25">
-      <c r="D4" t="s">
-        <v>570</v>
-      </c>
-      <c r="E4">
-        <v>1</v>
-      </c>
-      <c r="F4">
-        <v>2</v>
-      </c>
-      <c r="G4">
-        <v>3</v>
-      </c>
-      <c r="H4">
-        <v>4</v>
-      </c>
-      <c r="I4">
-        <v>5</v>
-      </c>
-      <c r="L4" t="s">
-        <v>579</v>
-      </c>
-    </row>
-    <row r="6" spans="4:13" x14ac:dyDescent="0.25">
-      <c r="D6" t="s">
-        <v>571</v>
-      </c>
-      <c r="L6" t="s">
-        <v>575</v>
-      </c>
-    </row>
-    <row r="7" spans="4:13" x14ac:dyDescent="0.25">
-      <c r="L7" t="s">
-        <v>576</v>
-      </c>
-    </row>
-    <row r="8" spans="4:13" x14ac:dyDescent="0.25">
-      <c r="E8" t="s">
-        <v>572</v>
-      </c>
-      <c r="I8" t="s">
-        <v>573</v>
-      </c>
-      <c r="L8" t="s">
-        <v>577</v>
-      </c>
-    </row>
-    <row r="9" spans="4:13" x14ac:dyDescent="0.25">
-      <c r="I9" t="s">
-        <v>574</v>
-      </c>
-    </row>
-    <row r="10" spans="4:13" x14ac:dyDescent="0.25">
-      <c r="I10" t="s">
-        <v>578</v>
-      </c>
-    </row>
-    <row r="12" spans="4:13" x14ac:dyDescent="0.25">
-      <c r="H12" t="s">
-        <v>580</v>
-      </c>
-      <c r="K12" t="s">
-        <v>587</v>
-      </c>
-    </row>
-    <row r="13" spans="4:13" x14ac:dyDescent="0.25">
-      <c r="H13" t="s">
-        <v>586</v>
-      </c>
-      <c r="K13" t="s">
-        <v>581</v>
-      </c>
-      <c r="L13" t="s">
-        <v>582</v>
-      </c>
-      <c r="M13" t="s">
-        <v>584</v>
-      </c>
-    </row>
-    <row r="14" spans="4:13" x14ac:dyDescent="0.25">
-      <c r="K14" t="s">
-        <v>183</v>
-      </c>
-      <c r="L14" t="s">
-        <v>583</v>
-      </c>
-      <c r="M14" t="s">
-        <v>585</v>
-      </c>
-    </row>
-    <row r="16" spans="4:13" x14ac:dyDescent="0.25">
-      <c r="K16" t="s">
-        <v>588</v>
-      </c>
-    </row>
-    <row r="100" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B100" t="s">
-        <v>569</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{913ED22E-69BE-48F7-94C8-6CAB8D4B66E4}">
-  <dimension ref="C99:C101"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="99" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C99" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="100" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C100" t="s">
-        <v>589</v>
-      </c>
-    </row>
-    <row r="101" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C101" t="s">
-        <v>590</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>